<commit_message>
Timesheet Updated and Submitted
</commit_message>
<xml_diff>
--- a/Documentation/Week 4/TimeSheet_Group21_Wk4.xlsx
+++ b/Documentation/Week 4/TimeSheet_Group21_Wk4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24432207_student_uwa_edu_au/Documents/UWA - Student/2026_Sem2/CITS3200 - Professional Computing/Project/Repo/CITS3200_Project/Documentation/Week 4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="207" documentId="8_{A2E391BD-BDDC-0249-A3FC-5E810E48BCB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A175852F-017B-47C5-B0ED-7C036DFAF580}"/>
+  <xr:revisionPtr revIDLastSave="223" documentId="8_{A2E391BD-BDDC-0249-A3FC-5E810E48BCB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BB7B378-492B-4554-BF72-1A3861F1F9EC}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="1" activeTab="1" xr2:uid="{62AB6E9C-1DC3-774E-B214-74EF319C3060}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="1" activeTab="2" xr2:uid="{62AB6E9C-1DC3-774E-B214-74EF319C3060}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="4" r:id="rId1"/>
@@ -1159,129 +1159,124 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1299,13 +1294,18 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1537,6 +1537,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1863,100 +1867,100 @@
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="90" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="82"/>
-      <c r="M1" s="82"/>
-      <c r="N1" s="82"/>
-      <c r="O1" s="82"/>
-      <c r="P1" s="82"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="86"/>
+      <c r="K1" s="86"/>
+      <c r="L1" s="86"/>
+      <c r="M1" s="86"/>
+      <c r="N1" s="86"/>
+      <c r="O1" s="86"/>
+      <c r="P1" s="86"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="81"/>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="82"/>
-      <c r="J2" s="82"/>
-      <c r="K2" s="82"/>
-      <c r="L2" s="82"/>
-      <c r="M2" s="82"/>
-      <c r="N2" s="82"/>
-      <c r="O2" s="82"/>
-      <c r="P2" s="82"/>
+      <c r="A2" s="89"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="86"/>
+      <c r="I2" s="86"/>
+      <c r="J2" s="86"/>
+      <c r="K2" s="86"/>
+      <c r="L2" s="86"/>
+      <c r="M2" s="86"/>
+      <c r="N2" s="86"/>
+      <c r="O2" s="86"/>
+      <c r="P2" s="86"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="81"/>
-      <c r="B3" s="81"/>
-      <c r="C3" s="81"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82"/>
-      <c r="K3" s="82"/>
-      <c r="L3" s="82"/>
-      <c r="M3" s="82"/>
-      <c r="N3" s="82"/>
-      <c r="O3" s="82"/>
-      <c r="P3" s="82"/>
+      <c r="A3" s="89"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="86"/>
+      <c r="G3" s="86"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="86"/>
+      <c r="K3" s="86"/>
+      <c r="L3" s="86"/>
+      <c r="M3" s="86"/>
+      <c r="N3" s="86"/>
+      <c r="O3" s="86"/>
+      <c r="P3" s="86"/>
     </row>
     <row r="4" spans="1:16" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A4" s="83" t="s">
+      <c r="A4" s="91" t="s">
         <v>76</v>
       </c>
-      <c r="B4" s="83"/>
-      <c r="C4" s="83"/>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
-      <c r="G4" s="83"/>
-      <c r="H4" s="83"/>
-      <c r="I4" s="83"/>
-      <c r="J4" s="83"/>
-      <c r="K4" s="83"/>
-      <c r="L4" s="83"/>
-      <c r="M4" s="83"/>
-      <c r="N4" s="83"/>
-      <c r="O4" s="83"/>
-      <c r="P4" s="83"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="91"/>
+      <c r="D4" s="91"/>
+      <c r="E4" s="91"/>
+      <c r="F4" s="91"/>
+      <c r="G4" s="91"/>
+      <c r="H4" s="91"/>
+      <c r="I4" s="91"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="91"/>
+      <c r="L4" s="91"/>
+      <c r="M4" s="91"/>
+      <c r="N4" s="91"/>
+      <c r="O4" s="91"/>
+      <c r="P4" s="91"/>
     </row>
     <row r="5" spans="1:16" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A5" s="83" t="s">
+      <c r="A5" s="91" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="83"/>
-      <c r="C5" s="83"/>
-      <c r="D5" s="83"/>
-      <c r="E5" s="83"/>
-      <c r="F5" s="83"/>
-      <c r="G5" s="83"/>
-      <c r="H5" s="83"/>
-      <c r="I5" s="83"/>
-      <c r="J5" s="83"/>
-      <c r="K5" s="83"/>
-      <c r="L5" s="83"/>
-      <c r="M5" s="83"/>
-      <c r="N5" s="83"/>
-      <c r="O5" s="83"/>
-      <c r="P5" s="83"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="91"/>
+      <c r="F5" s="91"/>
+      <c r="G5" s="91"/>
+      <c r="H5" s="91"/>
+      <c r="I5" s="91"/>
+      <c r="J5" s="91"/>
+      <c r="K5" s="91"/>
+      <c r="L5" s="91"/>
+      <c r="M5" s="91"/>
+      <c r="N5" s="91"/>
+      <c r="O5" s="91"/>
+      <c r="P5" s="91"/>
     </row>
     <row r="6" spans="1:16" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
@@ -1977,83 +1981,83 @@
       <c r="P6" s="8"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="85" t="s">
+      <c r="A7" s="93" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="85"/>
-      <c r="C7" s="85"/>
-      <c r="D7" s="85"/>
-      <c r="E7" s="86"/>
-      <c r="F7" s="86"/>
-      <c r="G7" s="86"/>
-      <c r="H7" s="86"/>
-      <c r="I7" s="86"/>
-      <c r="J7" s="86"/>
-      <c r="K7" s="86"/>
-      <c r="L7" s="86"/>
-      <c r="M7" s="86"/>
+      <c r="B7" s="93"/>
+      <c r="C7" s="93"/>
+      <c r="D7" s="93"/>
+      <c r="E7" s="94"/>
+      <c r="F7" s="94"/>
+      <c r="G7" s="94"/>
+      <c r="H7" s="94"/>
+      <c r="I7" s="94"/>
+      <c r="J7" s="94"/>
+      <c r="K7" s="94"/>
+      <c r="L7" s="94"/>
+      <c r="M7" s="94"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="84" t="s">
+      <c r="A8" s="92" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="84"/>
-      <c r="C8" s="84"/>
-      <c r="D8" s="84"/>
-      <c r="E8" s="84"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="84"/>
-      <c r="H8" s="84"/>
-      <c r="I8" s="84"/>
-      <c r="J8" s="84"/>
-      <c r="K8" s="84"/>
-      <c r="L8" s="84"/>
-      <c r="M8" s="84"/>
+      <c r="B8" s="92"/>
+      <c r="C8" s="92"/>
+      <c r="D8" s="92"/>
+      <c r="E8" s="92"/>
+      <c r="F8" s="92"/>
+      <c r="G8" s="92"/>
+      <c r="H8" s="92"/>
+      <c r="I8" s="92"/>
+      <c r="J8" s="92"/>
+      <c r="K8" s="92"/>
+      <c r="L8" s="92"/>
+      <c r="M8" s="92"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="84"/>
-      <c r="B9" s="84"/>
-      <c r="C9" s="84"/>
-      <c r="D9" s="84"/>
-      <c r="E9" s="84"/>
-      <c r="F9" s="84"/>
-      <c r="G9" s="84"/>
-      <c r="H9" s="84"/>
-      <c r="I9" s="84"/>
-      <c r="J9" s="84"/>
-      <c r="K9" s="84"/>
-      <c r="L9" s="84"/>
-      <c r="M9" s="84"/>
+      <c r="A9" s="92"/>
+      <c r="B9" s="92"/>
+      <c r="C9" s="92"/>
+      <c r="D9" s="92"/>
+      <c r="E9" s="92"/>
+      <c r="F9" s="92"/>
+      <c r="G9" s="92"/>
+      <c r="H9" s="92"/>
+      <c r="I9" s="92"/>
+      <c r="J9" s="92"/>
+      <c r="K9" s="92"/>
+      <c r="L9" s="92"/>
+      <c r="M9" s="92"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="84"/>
-      <c r="B10" s="84"/>
-      <c r="C10" s="84"/>
-      <c r="D10" s="84"/>
-      <c r="E10" s="84"/>
-      <c r="F10" s="84"/>
-      <c r="G10" s="84"/>
-      <c r="H10" s="84"/>
-      <c r="I10" s="84"/>
-      <c r="J10" s="84"/>
-      <c r="K10" s="84"/>
-      <c r="L10" s="84"/>
-      <c r="M10" s="84"/>
+      <c r="A10" s="92"/>
+      <c r="B10" s="92"/>
+      <c r="C10" s="92"/>
+      <c r="D10" s="92"/>
+      <c r="E10" s="92"/>
+      <c r="F10" s="92"/>
+      <c r="G10" s="92"/>
+      <c r="H10" s="92"/>
+      <c r="I10" s="92"/>
+      <c r="J10" s="92"/>
+      <c r="K10" s="92"/>
+      <c r="L10" s="92"/>
+      <c r="M10" s="92"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="84"/>
-      <c r="B11" s="84"/>
-      <c r="C11" s="84"/>
-      <c r="D11" s="84"/>
-      <c r="E11" s="84"/>
-      <c r="F11" s="84"/>
-      <c r="G11" s="84"/>
-      <c r="H11" s="84"/>
-      <c r="I11" s="84"/>
-      <c r="J11" s="84"/>
-      <c r="K11" s="84"/>
-      <c r="L11" s="84"/>
-      <c r="M11" s="84"/>
+      <c r="A11" s="92"/>
+      <c r="B11" s="92"/>
+      <c r="C11" s="92"/>
+      <c r="D11" s="92"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="92"/>
+      <c r="G11" s="92"/>
+      <c r="H11" s="92"/>
+      <c r="I11" s="92"/>
+      <c r="J11" s="92"/>
+      <c r="K11" s="92"/>
+      <c r="L11" s="92"/>
+      <c r="M11" s="92"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="53"/>
@@ -2071,187 +2075,187 @@
       <c r="M12" s="53"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="87" t="s">
+      <c r="A14" s="75" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="87"/>
-      <c r="C14" s="87"/>
-      <c r="D14" s="87"/>
-      <c r="E14" s="87"/>
-      <c r="F14" s="87"/>
-      <c r="G14" s="87"/>
-      <c r="H14" s="87"/>
-      <c r="I14" s="87"/>
-      <c r="J14" s="87"/>
-      <c r="K14" s="87"/>
-      <c r="L14" s="87"/>
-      <c r="M14" s="87"/>
+      <c r="B14" s="75"/>
+      <c r="C14" s="75"/>
+      <c r="D14" s="75"/>
+      <c r="E14" s="75"/>
+      <c r="F14" s="75"/>
+      <c r="G14" s="75"/>
+      <c r="H14" s="75"/>
+      <c r="I14" s="75"/>
+      <c r="J14" s="75"/>
+      <c r="K14" s="75"/>
+      <c r="L14" s="75"/>
+      <c r="M14" s="75"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="70" t="s">
+      <c r="A15" s="87" t="s">
         <v>80</v>
       </c>
-      <c r="B15" s="70"/>
-      <c r="C15" s="70"/>
-      <c r="D15" s="70"/>
-      <c r="E15" s="70"/>
-      <c r="F15" s="70"/>
-      <c r="G15" s="70"/>
-      <c r="H15" s="70"/>
-      <c r="I15" s="70"/>
-      <c r="J15" s="70"/>
-      <c r="K15" s="70"/>
-      <c r="L15" s="70"/>
-      <c r="M15" s="70"/>
+      <c r="B15" s="87"/>
+      <c r="C15" s="87"/>
+      <c r="D15" s="87"/>
+      <c r="E15" s="87"/>
+      <c r="F15" s="87"/>
+      <c r="G15" s="87"/>
+      <c r="H15" s="87"/>
+      <c r="I15" s="87"/>
+      <c r="J15" s="87"/>
+      <c r="K15" s="87"/>
+      <c r="L15" s="87"/>
+      <c r="M15" s="87"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="70"/>
-      <c r="B16" s="70"/>
-      <c r="C16" s="70"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="70"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="70"/>
-      <c r="H16" s="70"/>
-      <c r="I16" s="70"/>
-      <c r="J16" s="70"/>
-      <c r="K16" s="70"/>
-      <c r="L16" s="70"/>
-      <c r="M16" s="70"/>
+      <c r="A16" s="87"/>
+      <c r="B16" s="87"/>
+      <c r="C16" s="87"/>
+      <c r="D16" s="87"/>
+      <c r="E16" s="87"/>
+      <c r="F16" s="87"/>
+      <c r="G16" s="87"/>
+      <c r="H16" s="87"/>
+      <c r="I16" s="87"/>
+      <c r="J16" s="87"/>
+      <c r="K16" s="87"/>
+      <c r="L16" s="87"/>
+      <c r="M16" s="87"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" s="70" t="s">
+      <c r="A17" s="87" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="70"/>
-      <c r="C17" s="70"/>
-      <c r="D17" s="70"/>
-      <c r="E17" s="70"/>
-      <c r="F17" s="70"/>
-      <c r="G17" s="70"/>
-      <c r="H17" s="70"/>
-      <c r="I17" s="70"/>
-      <c r="J17" s="70"/>
-      <c r="K17" s="70"/>
-      <c r="L17" s="70"/>
-      <c r="M17" s="70"/>
+      <c r="B17" s="87"/>
+      <c r="C17" s="87"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="87"/>
+      <c r="F17" s="87"/>
+      <c r="G17" s="87"/>
+      <c r="H17" s="87"/>
+      <c r="I17" s="87"/>
+      <c r="J17" s="87"/>
+      <c r="K17" s="87"/>
+      <c r="L17" s="87"/>
+      <c r="M17" s="87"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" s="81"/>
-      <c r="B18" s="81"/>
-      <c r="C18" s="81"/>
-      <c r="D18" s="81"/>
-      <c r="E18" s="81"/>
-      <c r="F18" s="81"/>
-      <c r="G18" s="81"/>
-      <c r="H18" s="81"/>
-      <c r="I18" s="81"/>
-      <c r="J18" s="81"/>
-      <c r="K18" s="81"/>
-      <c r="L18" s="81"/>
-      <c r="M18" s="81"/>
+      <c r="A18" s="89"/>
+      <c r="B18" s="89"/>
+      <c r="C18" s="89"/>
+      <c r="D18" s="89"/>
+      <c r="E18" s="89"/>
+      <c r="F18" s="89"/>
+      <c r="G18" s="89"/>
+      <c r="H18" s="89"/>
+      <c r="I18" s="89"/>
+      <c r="J18" s="89"/>
+      <c r="K18" s="89"/>
+      <c r="L18" s="89"/>
+      <c r="M18" s="89"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="69" t="s">
+      <c r="A19" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="70"/>
-      <c r="C19" s="70"/>
-      <c r="D19" s="70"/>
-      <c r="E19" s="70"/>
-      <c r="F19" s="70"/>
-      <c r="G19" s="70"/>
-      <c r="H19" s="70"/>
-      <c r="I19" s="70"/>
-      <c r="J19" s="70"/>
-      <c r="K19" s="70"/>
-      <c r="L19" s="70"/>
-      <c r="M19" s="70"/>
+      <c r="B19" s="87"/>
+      <c r="C19" s="87"/>
+      <c r="D19" s="87"/>
+      <c r="E19" s="87"/>
+      <c r="F19" s="87"/>
+      <c r="G19" s="87"/>
+      <c r="H19" s="87"/>
+      <c r="I19" s="87"/>
+      <c r="J19" s="87"/>
+      <c r="K19" s="87"/>
+      <c r="L19" s="87"/>
+      <c r="M19" s="87"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="69" t="s">
+      <c r="A20" s="88" t="s">
         <v>82</v>
       </c>
-      <c r="B20" s="70"/>
-      <c r="C20" s="70"/>
-      <c r="D20" s="70"/>
-      <c r="E20" s="70"/>
-      <c r="F20" s="70"/>
-      <c r="G20" s="70"/>
-      <c r="H20" s="70"/>
-      <c r="I20" s="70"/>
-      <c r="J20" s="70"/>
-      <c r="K20" s="70"/>
-      <c r="L20" s="70"/>
-      <c r="M20" s="70"/>
+      <c r="B20" s="87"/>
+      <c r="C20" s="87"/>
+      <c r="D20" s="87"/>
+      <c r="E20" s="87"/>
+      <c r="F20" s="87"/>
+      <c r="G20" s="87"/>
+      <c r="H20" s="87"/>
+      <c r="I20" s="87"/>
+      <c r="J20" s="87"/>
+      <c r="K20" s="87"/>
+      <c r="L20" s="87"/>
+      <c r="M20" s="87"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="69" t="s">
+      <c r="A21" s="88" t="s">
         <v>83</v>
       </c>
-      <c r="B21" s="70"/>
-      <c r="C21" s="70"/>
-      <c r="D21" s="70"/>
-      <c r="E21" s="70"/>
-      <c r="F21" s="70"/>
-      <c r="G21" s="70"/>
-      <c r="H21" s="70"/>
-      <c r="I21" s="70"/>
-      <c r="J21" s="70"/>
-      <c r="K21" s="70"/>
-      <c r="L21" s="70"/>
-      <c r="M21" s="70"/>
+      <c r="B21" s="87"/>
+      <c r="C21" s="87"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="87"/>
+      <c r="F21" s="87"/>
+      <c r="G21" s="87"/>
+      <c r="H21" s="87"/>
+      <c r="I21" s="87"/>
+      <c r="J21" s="87"/>
+      <c r="K21" s="87"/>
+      <c r="L21" s="87"/>
+      <c r="M21" s="87"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="70" t="s">
+      <c r="A22" s="87" t="s">
         <v>86</v>
       </c>
-      <c r="B22" s="70"/>
-      <c r="C22" s="70"/>
-      <c r="D22" s="70"/>
-      <c r="E22" s="70"/>
-      <c r="F22" s="70"/>
-      <c r="G22" s="70"/>
-      <c r="H22" s="70"/>
-      <c r="I22" s="70"/>
-      <c r="J22" s="70"/>
-      <c r="K22" s="70"/>
-      <c r="L22" s="70"/>
-      <c r="M22" s="70"/>
+      <c r="B22" s="87"/>
+      <c r="C22" s="87"/>
+      <c r="D22" s="87"/>
+      <c r="E22" s="87"/>
+      <c r="F22" s="87"/>
+      <c r="G22" s="87"/>
+      <c r="H22" s="87"/>
+      <c r="I22" s="87"/>
+      <c r="J22" s="87"/>
+      <c r="K22" s="87"/>
+      <c r="L22" s="87"/>
+      <c r="M22" s="87"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="70" t="s">
+      <c r="A23" s="87" t="s">
         <v>85</v>
       </c>
-      <c r="B23" s="70"/>
-      <c r="C23" s="70"/>
-      <c r="D23" s="70"/>
-      <c r="E23" s="70"/>
-      <c r="F23" s="70"/>
-      <c r="G23" s="70"/>
-      <c r="H23" s="70"/>
-      <c r="I23" s="70"/>
-      <c r="J23" s="70"/>
-      <c r="K23" s="70"/>
-      <c r="L23" s="70"/>
-      <c r="M23" s="70"/>
+      <c r="B23" s="87"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="87"/>
+      <c r="E23" s="87"/>
+      <c r="F23" s="87"/>
+      <c r="G23" s="87"/>
+      <c r="H23" s="87"/>
+      <c r="I23" s="87"/>
+      <c r="J23" s="87"/>
+      <c r="K23" s="87"/>
+      <c r="L23" s="87"/>
+      <c r="M23" s="87"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="70" t="s">
+      <c r="A24" s="87" t="s">
         <v>84</v>
       </c>
-      <c r="B24" s="70"/>
-      <c r="C24" s="70"/>
-      <c r="D24" s="70"/>
-      <c r="E24" s="70"/>
-      <c r="F24" s="70"/>
-      <c r="G24" s="70"/>
-      <c r="H24" s="70"/>
-      <c r="I24" s="70"/>
-      <c r="J24" s="70"/>
-      <c r="K24" s="70"/>
-      <c r="L24" s="70"/>
-      <c r="M24" s="70"/>
+      <c r="B24" s="87"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="87"/>
+      <c r="E24" s="87"/>
+      <c r="F24" s="87"/>
+      <c r="G24" s="87"/>
+      <c r="H24" s="87"/>
+      <c r="I24" s="87"/>
+      <c r="J24" s="87"/>
+      <c r="K24" s="87"/>
+      <c r="L24" s="87"/>
+      <c r="M24" s="87"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="52"/>
@@ -2269,208 +2273,208 @@
       <c r="M25" s="52"/>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A27" s="73" t="s">
+      <c r="A27" s="98" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="73"/>
-      <c r="C27" s="73"/>
-      <c r="D27" s="73"/>
-      <c r="E27" s="67"/>
-      <c r="F27" s="67"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="67"/>
-      <c r="I27" s="67"/>
-      <c r="J27" s="67"/>
-      <c r="K27" s="67"/>
-      <c r="L27" s="67"/>
-      <c r="M27" s="67"/>
+      <c r="B27" s="98"/>
+      <c r="C27" s="98"/>
+      <c r="D27" s="98"/>
+      <c r="E27" s="99"/>
+      <c r="F27" s="99"/>
+      <c r="G27" s="99"/>
+      <c r="H27" s="99"/>
+      <c r="I27" s="99"/>
+      <c r="J27" s="99"/>
+      <c r="K27" s="99"/>
+      <c r="L27" s="99"/>
+      <c r="M27" s="99"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" s="74" t="s">
+      <c r="A28" s="82" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="75"/>
-      <c r="C28" s="75"/>
-      <c r="D28" s="75"/>
-      <c r="E28" s="75"/>
-      <c r="F28" s="75"/>
-      <c r="G28" s="75"/>
-      <c r="H28" s="75"/>
-      <c r="I28" s="75"/>
-      <c r="J28" s="75"/>
-      <c r="K28" s="75"/>
-      <c r="L28" s="75"/>
-      <c r="M28" s="75"/>
+      <c r="B28" s="100"/>
+      <c r="C28" s="100"/>
+      <c r="D28" s="100"/>
+      <c r="E28" s="100"/>
+      <c r="F28" s="100"/>
+      <c r="G28" s="100"/>
+      <c r="H28" s="100"/>
+      <c r="I28" s="100"/>
+      <c r="J28" s="100"/>
+      <c r="K28" s="100"/>
+      <c r="L28" s="100"/>
+      <c r="M28" s="100"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="76" t="s">
+      <c r="A29" s="80" t="s">
         <v>107</v>
       </c>
-      <c r="B29" s="76"/>
-      <c r="C29" s="76"/>
-      <c r="D29" s="76"/>
-      <c r="E29" s="88"/>
-      <c r="F29" s="88"/>
-      <c r="G29" s="88"/>
-      <c r="H29" s="88"/>
-      <c r="I29" s="88"/>
-      <c r="J29" s="88"/>
-      <c r="K29" s="88"/>
-      <c r="L29" s="88"/>
-      <c r="M29" s="88"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="83"/>
+      <c r="F29" s="83"/>
+      <c r="G29" s="83"/>
+      <c r="H29" s="83"/>
+      <c r="I29" s="83"/>
+      <c r="J29" s="83"/>
+      <c r="K29" s="83"/>
+      <c r="L29" s="83"/>
+      <c r="M29" s="83"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" s="76" t="s">
+      <c r="A30" s="80" t="s">
         <v>105</v>
       </c>
-      <c r="B30" s="76"/>
-      <c r="C30" s="76"/>
-      <c r="D30" s="76"/>
-      <c r="E30" s="77"/>
-      <c r="F30" s="77"/>
-      <c r="G30" s="77"/>
-      <c r="H30" s="77"/>
-      <c r="I30" s="77"/>
-      <c r="J30" s="77"/>
-      <c r="K30" s="77"/>
-      <c r="L30" s="77"/>
-      <c r="M30" s="77"/>
+      <c r="B30" s="80"/>
+      <c r="C30" s="80"/>
+      <c r="D30" s="80"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="81"/>
+      <c r="H30" s="81"/>
+      <c r="I30" s="81"/>
+      <c r="J30" s="81"/>
+      <c r="K30" s="81"/>
+      <c r="L30" s="81"/>
+      <c r="M30" s="81"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" s="76" t="s">
+      <c r="A31" s="80" t="s">
         <v>16</v>
       </c>
-      <c r="B31" s="82"/>
-      <c r="C31" s="82"/>
-      <c r="D31" s="82"/>
-      <c r="E31" s="82"/>
-      <c r="F31" s="82"/>
-      <c r="G31" s="82"/>
-      <c r="H31" s="82"/>
-      <c r="I31" s="82"/>
-      <c r="J31" s="82"/>
-      <c r="K31" s="82"/>
-      <c r="L31" s="82"/>
-      <c r="M31" s="82"/>
+      <c r="B31" s="86"/>
+      <c r="C31" s="86"/>
+      <c r="D31" s="86"/>
+      <c r="E31" s="86"/>
+      <c r="F31" s="86"/>
+      <c r="G31" s="86"/>
+      <c r="H31" s="86"/>
+      <c r="I31" s="86"/>
+      <c r="J31" s="86"/>
+      <c r="K31" s="86"/>
+      <c r="L31" s="86"/>
+      <c r="M31" s="86"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A32" s="76" t="s">
+      <c r="A32" s="80" t="s">
         <v>18</v>
       </c>
-      <c r="B32" s="76"/>
-      <c r="C32" s="76"/>
-      <c r="D32" s="76"/>
-      <c r="E32" s="77"/>
-      <c r="F32" s="77"/>
-      <c r="G32" s="77"/>
-      <c r="H32" s="77"/>
-      <c r="I32" s="77"/>
-      <c r="J32" s="77"/>
-      <c r="K32" s="77"/>
-      <c r="L32" s="77"/>
-      <c r="M32" s="77"/>
+      <c r="B32" s="80"/>
+      <c r="C32" s="80"/>
+      <c r="D32" s="80"/>
+      <c r="E32" s="81"/>
+      <c r="F32" s="81"/>
+      <c r="G32" s="81"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="81"/>
+      <c r="J32" s="81"/>
+      <c r="K32" s="81"/>
+      <c r="L32" s="81"/>
+      <c r="M32" s="81"/>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A33" s="74" t="s">
+      <c r="A33" s="82" t="s">
         <v>109</v>
       </c>
-      <c r="B33" s="74"/>
-      <c r="C33" s="74"/>
-      <c r="D33" s="74"/>
-      <c r="E33" s="77"/>
-      <c r="F33" s="77"/>
-      <c r="G33" s="77"/>
-      <c r="H33" s="77"/>
-      <c r="I33" s="77"/>
-      <c r="J33" s="77"/>
-      <c r="K33" s="77"/>
-      <c r="L33" s="77"/>
-      <c r="M33" s="77"/>
+      <c r="B33" s="82"/>
+      <c r="C33" s="82"/>
+      <c r="D33" s="82"/>
+      <c r="E33" s="81"/>
+      <c r="F33" s="81"/>
+      <c r="G33" s="81"/>
+      <c r="H33" s="81"/>
+      <c r="I33" s="81"/>
+      <c r="J33" s="81"/>
+      <c r="K33" s="81"/>
+      <c r="L33" s="81"/>
+      <c r="M33" s="81"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A34" s="76" t="s">
+      <c r="A34" s="80" t="s">
         <v>110</v>
       </c>
-      <c r="B34" s="76"/>
-      <c r="C34" s="76"/>
-      <c r="D34" s="76"/>
-      <c r="E34" s="77"/>
-      <c r="F34" s="77"/>
-      <c r="G34" s="77"/>
-      <c r="H34" s="77"/>
-      <c r="I34" s="77"/>
-      <c r="J34" s="77"/>
-      <c r="K34" s="77"/>
-      <c r="L34" s="77"/>
-      <c r="M34" s="77"/>
+      <c r="B34" s="80"/>
+      <c r="C34" s="80"/>
+      <c r="D34" s="80"/>
+      <c r="E34" s="81"/>
+      <c r="F34" s="81"/>
+      <c r="G34" s="81"/>
+      <c r="H34" s="81"/>
+      <c r="I34" s="81"/>
+      <c r="J34" s="81"/>
+      <c r="K34" s="81"/>
+      <c r="L34" s="81"/>
+      <c r="M34" s="81"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A35" s="74" t="s">
+      <c r="A35" s="82" t="s">
         <v>19</v>
       </c>
-      <c r="B35" s="74"/>
-      <c r="C35" s="74"/>
-      <c r="D35" s="74"/>
-      <c r="E35" s="77"/>
-      <c r="F35" s="77"/>
-      <c r="G35" s="77"/>
-      <c r="H35" s="77"/>
-      <c r="I35" s="77"/>
-      <c r="J35" s="77"/>
-      <c r="K35" s="77"/>
-      <c r="L35" s="77"/>
-      <c r="M35" s="77"/>
+      <c r="B35" s="82"/>
+      <c r="C35" s="82"/>
+      <c r="D35" s="82"/>
+      <c r="E35" s="81"/>
+      <c r="F35" s="81"/>
+      <c r="G35" s="81"/>
+      <c r="H35" s="81"/>
+      <c r="I35" s="81"/>
+      <c r="J35" s="81"/>
+      <c r="K35" s="81"/>
+      <c r="L35" s="81"/>
+      <c r="M35" s="81"/>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A36" s="74" t="s">
+      <c r="A36" s="82" t="s">
         <v>20</v>
       </c>
-      <c r="B36" s="74"/>
-      <c r="C36" s="74"/>
-      <c r="D36" s="74"/>
-      <c r="E36" s="77"/>
-      <c r="F36" s="77"/>
-      <c r="G36" s="77"/>
-      <c r="H36" s="77"/>
-      <c r="I36" s="77"/>
-      <c r="J36" s="77"/>
-      <c r="K36" s="77"/>
-      <c r="L36" s="77"/>
-      <c r="M36" s="77"/>
+      <c r="B36" s="82"/>
+      <c r="C36" s="82"/>
+      <c r="D36" s="82"/>
+      <c r="E36" s="81"/>
+      <c r="F36" s="81"/>
+      <c r="G36" s="81"/>
+      <c r="H36" s="81"/>
+      <c r="I36" s="81"/>
+      <c r="J36" s="81"/>
+      <c r="K36" s="81"/>
+      <c r="L36" s="81"/>
+      <c r="M36" s="81"/>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A37" s="74" t="s">
+      <c r="A37" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="B37" s="74"/>
-      <c r="C37" s="74"/>
-      <c r="D37" s="74"/>
-      <c r="E37" s="77"/>
-      <c r="F37" s="77"/>
-      <c r="G37" s="77"/>
-      <c r="H37" s="77"/>
-      <c r="I37" s="77"/>
-      <c r="J37" s="77"/>
-      <c r="K37" s="77"/>
-      <c r="L37" s="77"/>
-      <c r="M37" s="77"/>
+      <c r="B37" s="82"/>
+      <c r="C37" s="82"/>
+      <c r="D37" s="82"/>
+      <c r="E37" s="81"/>
+      <c r="F37" s="81"/>
+      <c r="G37" s="81"/>
+      <c r="H37" s="81"/>
+      <c r="I37" s="81"/>
+      <c r="J37" s="81"/>
+      <c r="K37" s="81"/>
+      <c r="L37" s="81"/>
+      <c r="M37" s="81"/>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A38" s="74" t="s">
+      <c r="A38" s="82" t="s">
         <v>45</v>
       </c>
-      <c r="B38" s="67"/>
-      <c r="C38" s="67"/>
-      <c r="D38" s="67"/>
-      <c r="E38" s="67"/>
-      <c r="F38" s="67"/>
-      <c r="G38" s="67"/>
-      <c r="H38" s="67"/>
-      <c r="I38" s="67"/>
-      <c r="J38" s="67"/>
-      <c r="K38" s="67"/>
-      <c r="L38" s="67"/>
-      <c r="M38" s="67"/>
+      <c r="B38" s="99"/>
+      <c r="C38" s="99"/>
+      <c r="D38" s="99"/>
+      <c r="E38" s="99"/>
+      <c r="F38" s="99"/>
+      <c r="G38" s="99"/>
+      <c r="H38" s="99"/>
+      <c r="I38" s="99"/>
+      <c r="J38" s="99"/>
+      <c r="K38" s="99"/>
+      <c r="L38" s="99"/>
+      <c r="M38" s="99"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="51"/>
@@ -2488,38 +2492,38 @@
       <c r="M39" s="59"/>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A41" s="89" t="s">
+      <c r="A41" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="B41" s="90"/>
-      <c r="C41" s="90"/>
-      <c r="D41" s="90"/>
-      <c r="E41" s="90"/>
-      <c r="F41" s="90"/>
-      <c r="G41" s="90"/>
-      <c r="H41" s="90"/>
-      <c r="I41" s="90"/>
-      <c r="J41" s="90"/>
-      <c r="K41" s="90"/>
-      <c r="L41" s="90"/>
-      <c r="M41" s="90"/>
+      <c r="B41" s="85"/>
+      <c r="C41" s="85"/>
+      <c r="D41" s="85"/>
+      <c r="E41" s="85"/>
+      <c r="F41" s="85"/>
+      <c r="G41" s="85"/>
+      <c r="H41" s="85"/>
+      <c r="I41" s="85"/>
+      <c r="J41" s="85"/>
+      <c r="K41" s="85"/>
+      <c r="L41" s="85"/>
+      <c r="M41" s="85"/>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A42" s="66" t="s">
+      <c r="A42" s="102" t="s">
         <v>26</v>
       </c>
-      <c r="B42" s="67"/>
-      <c r="C42" s="67"/>
-      <c r="D42" s="67"/>
-      <c r="E42" s="67"/>
-      <c r="F42" s="67"/>
-      <c r="G42" s="67"/>
-      <c r="H42" s="67"/>
-      <c r="I42" s="67"/>
-      <c r="J42" s="67"/>
-      <c r="K42" s="67"/>
-      <c r="L42" s="67"/>
-      <c r="M42" s="67"/>
+      <c r="B42" s="99"/>
+      <c r="C42" s="99"/>
+      <c r="D42" s="99"/>
+      <c r="E42" s="99"/>
+      <c r="F42" s="99"/>
+      <c r="G42" s="99"/>
+      <c r="H42" s="99"/>
+      <c r="I42" s="99"/>
+      <c r="J42" s="99"/>
+      <c r="K42" s="99"/>
+      <c r="L42" s="99"/>
+      <c r="M42" s="99"/>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="50"/>
@@ -2542,106 +2546,106 @@
       <c r="C44" s="7"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A45" s="71" t="s">
+      <c r="A45" s="96" t="s">
         <v>29</v>
       </c>
-      <c r="B45" s="72"/>
-      <c r="C45" s="72"/>
-      <c r="D45" s="72"/>
-      <c r="E45" s="72"/>
-      <c r="F45" s="72"/>
-      <c r="G45" s="72"/>
-      <c r="H45" s="72"/>
-      <c r="I45" s="72"/>
-      <c r="J45" s="72"/>
-      <c r="K45" s="72"/>
-      <c r="L45" s="72"/>
-      <c r="M45" s="72"/>
+      <c r="B45" s="97"/>
+      <c r="C45" s="97"/>
+      <c r="D45" s="97"/>
+      <c r="E45" s="97"/>
+      <c r="F45" s="97"/>
+      <c r="G45" s="97"/>
+      <c r="H45" s="97"/>
+      <c r="I45" s="97"/>
+      <c r="J45" s="97"/>
+      <c r="K45" s="97"/>
+      <c r="L45" s="97"/>
+      <c r="M45" s="97"/>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A46" s="79" t="s">
+      <c r="A46" s="103" t="s">
         <v>30</v>
       </c>
-      <c r="B46" s="79"/>
-      <c r="C46" s="79"/>
-      <c r="D46" s="79"/>
-      <c r="E46" s="79"/>
-      <c r="F46" s="79"/>
-      <c r="G46" s="79"/>
-      <c r="H46" s="79"/>
-      <c r="I46" s="79"/>
-      <c r="J46" s="79"/>
-      <c r="K46" s="79"/>
-      <c r="L46" s="79"/>
-      <c r="M46" s="79"/>
+      <c r="B46" s="103"/>
+      <c r="C46" s="103"/>
+      <c r="D46" s="103"/>
+      <c r="E46" s="103"/>
+      <c r="F46" s="103"/>
+      <c r="G46" s="103"/>
+      <c r="H46" s="103"/>
+      <c r="I46" s="103"/>
+      <c r="J46" s="103"/>
+      <c r="K46" s="103"/>
+      <c r="L46" s="103"/>
+      <c r="M46" s="103"/>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A47" s="79" t="s">
+      <c r="A47" s="103" t="s">
         <v>52</v>
       </c>
-      <c r="B47" s="79"/>
-      <c r="C47" s="79"/>
-      <c r="D47" s="79"/>
-      <c r="E47" s="79"/>
-      <c r="F47" s="79"/>
-      <c r="G47" s="79"/>
-      <c r="H47" s="79"/>
-      <c r="I47" s="79"/>
-      <c r="J47" s="79"/>
-      <c r="K47" s="79"/>
-      <c r="L47" s="79"/>
-      <c r="M47" s="79"/>
+      <c r="B47" s="103"/>
+      <c r="C47" s="103"/>
+      <c r="D47" s="103"/>
+      <c r="E47" s="103"/>
+      <c r="F47" s="103"/>
+      <c r="G47" s="103"/>
+      <c r="H47" s="103"/>
+      <c r="I47" s="103"/>
+      <c r="J47" s="103"/>
+      <c r="K47" s="103"/>
+      <c r="L47" s="103"/>
+      <c r="M47" s="103"/>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A48" s="79" t="s">
+      <c r="A48" s="103" t="s">
         <v>53</v>
       </c>
-      <c r="B48" s="79"/>
-      <c r="C48" s="79"/>
-      <c r="D48" s="79"/>
-      <c r="E48" s="79"/>
-      <c r="F48" s="79"/>
-      <c r="G48" s="79"/>
-      <c r="H48" s="79"/>
-      <c r="I48" s="79"/>
-      <c r="J48" s="79"/>
-      <c r="K48" s="79"/>
-      <c r="L48" s="79"/>
-      <c r="M48" s="79"/>
+      <c r="B48" s="103"/>
+      <c r="C48" s="103"/>
+      <c r="D48" s="103"/>
+      <c r="E48" s="103"/>
+      <c r="F48" s="103"/>
+      <c r="G48" s="103"/>
+      <c r="H48" s="103"/>
+      <c r="I48" s="103"/>
+      <c r="J48" s="103"/>
+      <c r="K48" s="103"/>
+      <c r="L48" s="103"/>
+      <c r="M48" s="103"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A49" s="78" t="s">
+      <c r="A49" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="B49" s="78"/>
-      <c r="C49" s="78"/>
-      <c r="D49" s="78"/>
-      <c r="E49" s="78"/>
-      <c r="F49" s="78"/>
-      <c r="G49" s="78"/>
-      <c r="H49" s="78"/>
-      <c r="I49" s="78"/>
-      <c r="J49" s="78"/>
-      <c r="K49" s="78"/>
-      <c r="L49" s="78"/>
-      <c r="M49" s="78"/>
+      <c r="B49" s="101"/>
+      <c r="C49" s="101"/>
+      <c r="D49" s="101"/>
+      <c r="E49" s="101"/>
+      <c r="F49" s="101"/>
+      <c r="G49" s="101"/>
+      <c r="H49" s="101"/>
+      <c r="I49" s="101"/>
+      <c r="J49" s="101"/>
+      <c r="K49" s="101"/>
+      <c r="L49" s="101"/>
+      <c r="M49" s="101"/>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A50" s="78" t="s">
+      <c r="A50" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="B50" s="78"/>
-      <c r="C50" s="78"/>
-      <c r="D50" s="78"/>
-      <c r="E50" s="78"/>
-      <c r="F50" s="78"/>
-      <c r="G50" s="78"/>
-      <c r="H50" s="78"/>
-      <c r="I50" s="78"/>
-      <c r="J50" s="78"/>
-      <c r="K50" s="78"/>
-      <c r="L50" s="78"/>
-      <c r="M50" s="78"/>
+      <c r="B50" s="101"/>
+      <c r="C50" s="101"/>
+      <c r="D50" s="101"/>
+      <c r="E50" s="101"/>
+      <c r="F50" s="101"/>
+      <c r="G50" s="101"/>
+      <c r="H50" s="101"/>
+      <c r="I50" s="101"/>
+      <c r="J50" s="101"/>
+      <c r="K50" s="101"/>
+      <c r="L50" s="101"/>
+      <c r="M50" s="101"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="55"/>
@@ -2689,100 +2693,81 @@
       <c r="M53" s="58"/>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A54" s="68" t="s">
+      <c r="A54" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="B54" s="68"/>
-      <c r="C54" s="68"/>
-      <c r="D54" s="68"/>
-      <c r="E54" s="68"/>
-      <c r="F54" s="68"/>
-      <c r="G54" s="68"/>
-      <c r="H54" s="68"/>
-      <c r="I54" s="68"/>
-      <c r="J54" s="68"/>
-      <c r="K54" s="68"/>
-      <c r="L54" s="68"/>
-      <c r="M54" s="68"/>
-      <c r="N54" s="68"/>
-      <c r="O54" s="68"/>
-      <c r="P54" s="68"/>
+      <c r="B54" s="95"/>
+      <c r="C54" s="95"/>
+      <c r="D54" s="95"/>
+      <c r="E54" s="95"/>
+      <c r="F54" s="95"/>
+      <c r="G54" s="95"/>
+      <c r="H54" s="95"/>
+      <c r="I54" s="95"/>
+      <c r="J54" s="95"/>
+      <c r="K54" s="95"/>
+      <c r="L54" s="95"/>
+      <c r="M54" s="95"/>
+      <c r="N54" s="95"/>
+      <c r="O54" s="95"/>
+      <c r="P54" s="95"/>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A55" s="68"/>
-      <c r="B55" s="68"/>
-      <c r="C55" s="68"/>
-      <c r="D55" s="68"/>
-      <c r="E55" s="68"/>
-      <c r="F55" s="68"/>
-      <c r="G55" s="68"/>
-      <c r="H55" s="68"/>
-      <c r="I55" s="68"/>
-      <c r="J55" s="68"/>
-      <c r="K55" s="68"/>
-      <c r="L55" s="68"/>
-      <c r="M55" s="68"/>
-      <c r="N55" s="68"/>
-      <c r="O55" s="68"/>
-      <c r="P55" s="68"/>
+      <c r="A55" s="95"/>
+      <c r="B55" s="95"/>
+      <c r="C55" s="95"/>
+      <c r="D55" s="95"/>
+      <c r="E55" s="95"/>
+      <c r="F55" s="95"/>
+      <c r="G55" s="95"/>
+      <c r="H55" s="95"/>
+      <c r="I55" s="95"/>
+      <c r="J55" s="95"/>
+      <c r="K55" s="95"/>
+      <c r="L55" s="95"/>
+      <c r="M55" s="95"/>
+      <c r="N55" s="95"/>
+      <c r="O55" s="95"/>
+      <c r="P55" s="95"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A56" s="68"/>
-      <c r="B56" s="68"/>
-      <c r="C56" s="68"/>
-      <c r="D56" s="68"/>
-      <c r="E56" s="68"/>
-      <c r="F56" s="68"/>
-      <c r="G56" s="68"/>
-      <c r="H56" s="68"/>
-      <c r="I56" s="68"/>
-      <c r="J56" s="68"/>
-      <c r="K56" s="68"/>
-      <c r="L56" s="68"/>
-      <c r="M56" s="68"/>
-      <c r="N56" s="68"/>
-      <c r="O56" s="68"/>
-      <c r="P56" s="68"/>
+      <c r="A56" s="95"/>
+      <c r="B56" s="95"/>
+      <c r="C56" s="95"/>
+      <c r="D56" s="95"/>
+      <c r="E56" s="95"/>
+      <c r="F56" s="95"/>
+      <c r="G56" s="95"/>
+      <c r="H56" s="95"/>
+      <c r="I56" s="95"/>
+      <c r="J56" s="95"/>
+      <c r="K56" s="95"/>
+      <c r="L56" s="95"/>
+      <c r="M56" s="95"/>
+      <c r="N56" s="95"/>
+      <c r="O56" s="95"/>
+      <c r="P56" s="95"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A57" s="68"/>
-      <c r="B57" s="68"/>
-      <c r="C57" s="68"/>
-      <c r="D57" s="68"/>
-      <c r="E57" s="68"/>
-      <c r="F57" s="68"/>
-      <c r="G57" s="68"/>
-      <c r="H57" s="68"/>
-      <c r="I57" s="68"/>
-      <c r="J57" s="68"/>
-      <c r="K57" s="68"/>
-      <c r="L57" s="68"/>
-      <c r="M57" s="68"/>
-      <c r="N57" s="68"/>
-      <c r="O57" s="68"/>
-      <c r="P57" s="68"/>
+      <c r="A57" s="95"/>
+      <c r="B57" s="95"/>
+      <c r="C57" s="95"/>
+      <c r="D57" s="95"/>
+      <c r="E57" s="95"/>
+      <c r="F57" s="95"/>
+      <c r="G57" s="95"/>
+      <c r="H57" s="95"/>
+      <c r="I57" s="95"/>
+      <c r="J57" s="95"/>
+      <c r="K57" s="95"/>
+      <c r="L57" s="95"/>
+      <c r="M57" s="95"/>
+      <c r="N57" s="95"/>
+      <c r="O57" s="95"/>
+      <c r="P57" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A30:M30"/>
-    <mergeCell ref="A32:M32"/>
-    <mergeCell ref="A33:M33"/>
-    <mergeCell ref="A29:M29"/>
-    <mergeCell ref="A41:M41"/>
-    <mergeCell ref="A35:M35"/>
-    <mergeCell ref="A36:M36"/>
-    <mergeCell ref="A37:M37"/>
-    <mergeCell ref="A31:M31"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A15:M16"/>
-    <mergeCell ref="A19:M19"/>
-    <mergeCell ref="A20:M20"/>
-    <mergeCell ref="A17:M18"/>
-    <mergeCell ref="A1:P3"/>
-    <mergeCell ref="A4:P4"/>
-    <mergeCell ref="A8:M11"/>
-    <mergeCell ref="A7:M7"/>
-    <mergeCell ref="A5:P5"/>
     <mergeCell ref="A54:P57"/>
     <mergeCell ref="A21:M21"/>
     <mergeCell ref="A22:M22"/>
@@ -2799,6 +2784,25 @@
     <mergeCell ref="A47:M47"/>
     <mergeCell ref="A48:M48"/>
     <mergeCell ref="A49:M49"/>
+    <mergeCell ref="A1:P3"/>
+    <mergeCell ref="A4:P4"/>
+    <mergeCell ref="A8:M11"/>
+    <mergeCell ref="A7:M7"/>
+    <mergeCell ref="A5:P5"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A15:M16"/>
+    <mergeCell ref="A19:M19"/>
+    <mergeCell ref="A20:M20"/>
+    <mergeCell ref="A17:M18"/>
+    <mergeCell ref="A30:M30"/>
+    <mergeCell ref="A32:M32"/>
+    <mergeCell ref="A33:M33"/>
+    <mergeCell ref="A29:M29"/>
+    <mergeCell ref="A41:M41"/>
+    <mergeCell ref="A35:M35"/>
+    <mergeCell ref="A36:M36"/>
+    <mergeCell ref="A37:M37"/>
+    <mergeCell ref="A31:M31"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2823,11 +2827,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="75" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -2842,11 +2846,11 @@
       <c r="Q1" s="2"/>
     </row>
     <row r="2" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
       <c r="D2" s="10"/>
       <c r="E2" s="10"/>
       <c r="F2" s="11"/>
@@ -2863,11 +2867,11 @@
       <c r="Q2" s="2"/>
     </row>
     <row r="3" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="92" t="s">
+      <c r="A3" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="92"/>
-      <c r="C3" s="92"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
       <c r="F3" s="12"/>
@@ -2884,11 +2888,11 @@
       <c r="Q3" s="3"/>
     </row>
     <row r="4" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="92" t="s">
+      <c r="A4" s="76" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="92"/>
-      <c r="C4" s="92"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
       <c r="D4" s="12"/>
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
@@ -2905,11 +2909,11 @@
       <c r="Q4" s="4"/>
     </row>
     <row r="5" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="92" t="s">
+      <c r="A5" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="92"/>
-      <c r="C5" s="92"/>
+      <c r="B5" s="76"/>
+      <c r="C5" s="76"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="5"/>
@@ -2926,11 +2930,11 @@
       <c r="Q5" s="5"/>
     </row>
     <row r="6" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="87" t="s">
+      <c r="A6" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="87"/>
-      <c r="C6" s="87"/>
+      <c r="B6" s="75"/>
+      <c r="C6" s="75"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="5"/>
@@ -2947,11 +2951,11 @@
       <c r="Q6" s="5"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A7" s="87" t="s">
+      <c r="A7" s="75" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="87"/>
-      <c r="C7" s="87"/>
+      <c r="B7" s="75"/>
+      <c r="C7" s="75"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="5"/>
@@ -2987,102 +2991,102 @@
       <c r="Q8" s="5"/>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A9" s="93" t="s">
-        <v>0</v>
-      </c>
-      <c r="B9" s="94"/>
+      <c r="A9" s="77" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="78"/>
       <c r="C9" s="54">
         <v>360</v>
       </c>
     </row>
     <row r="10" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="96" t="s">
+      <c r="A10" s="67" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="96"/>
+      <c r="B10" s="67"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="97" t="s">
+      <c r="D10" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="E10" s="98"/>
-      <c r="F10" s="98"/>
-      <c r="G10" s="98"/>
-      <c r="H10" s="98"/>
-      <c r="I10" s="98"/>
-      <c r="J10" s="98"/>
-      <c r="K10" s="98"/>
-      <c r="L10" s="98"/>
-      <c r="M10" s="98"/>
-      <c r="N10" s="99"/>
-      <c r="O10" s="99"/>
-      <c r="P10" s="99"/>
-      <c r="Q10" s="99"/>
-      <c r="R10" s="99"/>
-      <c r="S10" s="99"/>
-      <c r="T10" s="99"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="69"/>
+      <c r="H10" s="69"/>
+      <c r="I10" s="69"/>
+      <c r="J10" s="69"/>
+      <c r="K10" s="69"/>
+      <c r="L10" s="69"/>
+      <c r="M10" s="69"/>
+      <c r="N10" s="70"/>
+      <c r="O10" s="70"/>
+      <c r="P10" s="70"/>
+      <c r="Q10" s="70"/>
+      <c r="R10" s="70"/>
+      <c r="S10" s="70"/>
+      <c r="T10" s="70"/>
       <c r="U10" s="13"/>
       <c r="V10" s="13"/>
       <c r="W10" s="13"/>
       <c r="X10" s="13"/>
     </row>
     <row r="11" spans="1:24" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="100" t="s">
+      <c r="A11" s="71" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="101" t="s">
+      <c r="B11" s="72" t="s">
         <v>60</v>
       </c>
-      <c r="C11" s="102" t="s">
+      <c r="C11" s="73" t="s">
         <v>108</v>
       </c>
-      <c r="D11" s="91" t="s">
+      <c r="D11" s="66" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="91"/>
-      <c r="F11" s="91" t="s">
+      <c r="E11" s="66"/>
+      <c r="F11" s="66" t="s">
         <v>62</v>
       </c>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91" t="s">
+      <c r="G11" s="66"/>
+      <c r="H11" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91" t="s">
+      <c r="I11" s="66"/>
+      <c r="J11" s="66" t="s">
         <v>64</v>
       </c>
-      <c r="K11" s="91"/>
-      <c r="L11" s="91" t="s">
+      <c r="K11" s="66"/>
+      <c r="L11" s="66" t="s">
         <v>65</v>
       </c>
-      <c r="M11" s="91"/>
-      <c r="N11" s="91" t="s">
+      <c r="M11" s="66"/>
+      <c r="N11" s="66" t="s">
         <v>66</v>
       </c>
-      <c r="O11" s="91"/>
-      <c r="P11" s="91" t="s">
+      <c r="O11" s="66"/>
+      <c r="P11" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="Q11" s="91"/>
-      <c r="R11" s="91" t="s">
+      <c r="Q11" s="66"/>
+      <c r="R11" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="S11" s="91"/>
-      <c r="T11" s="91" t="s">
+      <c r="S11" s="66"/>
+      <c r="T11" s="66" t="s">
         <v>71</v>
       </c>
-      <c r="U11" s="91"/>
-      <c r="V11" s="91" t="s">
+      <c r="U11" s="66"/>
+      <c r="V11" s="66" t="s">
         <v>72</v>
       </c>
-      <c r="W11" s="91"/>
+      <c r="W11" s="66"/>
       <c r="X11" s="14" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:24" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="100"/>
-      <c r="B12" s="101"/>
-      <c r="C12" s="103"/>
+      <c r="A12" s="71"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="74"/>
       <c r="D12" s="15" t="s">
         <v>68</v>
       </c>
@@ -3529,7 +3533,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="19">
-        <v>4.75</v>
+        <v>7.75</v>
       </c>
       <c r="J23" s="18"/>
       <c r="K23" s="19"/>
@@ -3747,7 +3751,7 @@
       </c>
       <c r="I30" s="56">
         <f t="shared" si="0"/>
-        <v>28.25</v>
+        <v>31.25</v>
       </c>
       <c r="J30" s="56">
         <f t="shared" si="0"/>
@@ -3857,11 +3861,15 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="V11:W11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="R11:S11"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A7:C7"/>
     <mergeCell ref="J11:K11"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="D10:T10"/>
@@ -3871,15 +3879,11 @@
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="C11:C12"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="V11:W11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="P11:Q11"/>
+    <mergeCell ref="R11:S11"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3910,30 +3914,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="98" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
+      <c r="B1" s="98"/>
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
       <c r="E1" s="22"/>
     </row>
     <row r="2" spans="1:47" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A2" s="105" t="s">
+      <c r="A2" s="107" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="105"/>
-      <c r="C2" s="105"/>
-      <c r="D2" s="105"/>
+      <c r="B2" s="107"/>
+      <c r="C2" s="107"/>
+      <c r="D2" s="107"/>
       <c r="E2" s="23"/>
     </row>
     <row r="3" spans="1:47" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A3" s="105" t="s">
+      <c r="A3" s="107" t="s">
         <v>105</v>
       </c>
-      <c r="B3" s="105"/>
-      <c r="C3" s="105"/>
-      <c r="D3" s="105"/>
+      <c r="B3" s="107"/>
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
       <c r="E3" s="23"/>
     </row>
     <row r="4" spans="1:47" ht="13.8" x14ac:dyDescent="0.25">
@@ -3946,139 +3950,139 @@
       <c r="E4" s="23"/>
     </row>
     <row r="5" spans="1:47" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A5" s="105" t="s">
+      <c r="A5" s="107" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="105"/>
-      <c r="C5" s="105"/>
-      <c r="D5" s="105"/>
+      <c r="B5" s="107"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="107"/>
       <c r="E5" s="23"/>
     </row>
     <row r="6" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A6" s="73" t="s">
+      <c r="A6" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="73"/>
-      <c r="C6" s="73"/>
-      <c r="D6" s="73"/>
+      <c r="B6" s="98"/>
+      <c r="C6" s="98"/>
+      <c r="D6" s="98"/>
       <c r="E6" s="22"/>
     </row>
     <row r="7" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A7" s="105" t="s">
+      <c r="A7" s="107" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="105"/>
-      <c r="C7" s="105"/>
-      <c r="D7" s="105"/>
+      <c r="B7" s="107"/>
+      <c r="C7" s="107"/>
+      <c r="D7" s="107"/>
       <c r="E7" s="22"/>
     </row>
     <row r="8" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A8" s="73" t="s">
+      <c r="A8" s="98" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="73"/>
-      <c r="C8" s="73"/>
-      <c r="D8" s="73"/>
+      <c r="B8" s="98"/>
+      <c r="C8" s="98"/>
+      <c r="D8" s="98"/>
       <c r="E8" s="22"/>
     </row>
     <row r="9" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A9" s="73" t="s">
+      <c r="A9" s="98" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="73"/>
-      <c r="C9" s="73"/>
-      <c r="D9" s="73"/>
+      <c r="B9" s="98"/>
+      <c r="C9" s="98"/>
+      <c r="D9" s="98"/>
       <c r="E9" s="22"/>
     </row>
     <row r="10" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A10" s="73" t="s">
+      <c r="A10" s="98" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="73"/>
-      <c r="C10" s="73"/>
-      <c r="D10" s="73"/>
+      <c r="B10" s="98"/>
+      <c r="C10" s="98"/>
+      <c r="D10" s="98"/>
       <c r="E10" s="22"/>
     </row>
     <row r="11" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A11" s="73" t="s">
+      <c r="A11" s="98" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="73"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="73"/>
+      <c r="B11" s="98"/>
+      <c r="C11" s="98"/>
+      <c r="D11" s="98"/>
       <c r="E11" s="22"/>
     </row>
     <row r="12" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A12" s="73"/>
-      <c r="B12" s="73"/>
-      <c r="C12" s="73"/>
-      <c r="D12" s="73"/>
+      <c r="A12" s="98"/>
+      <c r="B12" s="98"/>
+      <c r="C12" s="98"/>
+      <c r="D12" s="98"/>
       <c r="E12" s="22"/>
     </row>
     <row r="13" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A13" s="112" t="str">
+      <c r="A13" s="111" t="str">
         <f>IF(AND(COUNT(D17:D68) &gt;0,(D69&lt;&gt;100)),"Value does not sum to $100","Value is OK")</f>
         <v>Value is OK</v>
       </c>
-      <c r="B13" s="113"/>
-      <c r="C13" s="113"/>
-      <c r="D13" s="114"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="113"/>
     </row>
     <row r="14" spans="1:47" s="21" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="65" t="s">
+      <c r="A14" s="114" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="65" t="s">
+      <c r="B14" s="114" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="65" t="s">
+      <c r="C14" s="114" t="s">
         <v>108</v>
       </c>
-      <c r="D14" s="65" t="s">
+      <c r="D14" s="114" t="s">
         <v>102</v>
       </c>
-      <c r="E14" s="109" t="s">
+      <c r="E14" s="108" t="s">
         <v>103</v>
       </c>
-      <c r="F14" s="110"/>
-      <c r="G14" s="110"/>
-      <c r="H14" s="110"/>
-      <c r="I14" s="110"/>
-      <c r="J14" s="110"/>
-      <c r="K14" s="110"/>
-      <c r="L14" s="110"/>
-      <c r="M14" s="110"/>
-      <c r="N14" s="110"/>
-      <c r="O14" s="110"/>
-      <c r="P14" s="110"/>
-      <c r="Q14" s="110"/>
-      <c r="R14" s="110"/>
-      <c r="S14" s="110"/>
-      <c r="T14" s="110"/>
-      <c r="U14" s="110"/>
-      <c r="V14" s="110"/>
-      <c r="W14" s="110"/>
-      <c r="X14" s="110"/>
-      <c r="Y14" s="110"/>
-      <c r="Z14" s="110"/>
-      <c r="AA14" s="110"/>
-      <c r="AB14" s="110"/>
-      <c r="AC14" s="110"/>
-      <c r="AD14" s="110"/>
-      <c r="AE14" s="110"/>
-      <c r="AF14" s="110"/>
-      <c r="AG14" s="110"/>
-      <c r="AH14" s="110"/>
-      <c r="AI14" s="110"/>
-      <c r="AJ14" s="110"/>
-      <c r="AK14" s="110"/>
-      <c r="AL14" s="110"/>
-      <c r="AM14" s="110"/>
-      <c r="AN14" s="110"/>
-      <c r="AO14" s="110"/>
-      <c r="AP14" s="110"/>
-      <c r="AQ14" s="110"/>
-      <c r="AR14" s="111"/>
+      <c r="F14" s="109"/>
+      <c r="G14" s="109"/>
+      <c r="H14" s="109"/>
+      <c r="I14" s="109"/>
+      <c r="J14" s="109"/>
+      <c r="K14" s="109"/>
+      <c r="L14" s="109"/>
+      <c r="M14" s="109"/>
+      <c r="N14" s="109"/>
+      <c r="O14" s="109"/>
+      <c r="P14" s="109"/>
+      <c r="Q14" s="109"/>
+      <c r="R14" s="109"/>
+      <c r="S14" s="109"/>
+      <c r="T14" s="109"/>
+      <c r="U14" s="109"/>
+      <c r="V14" s="109"/>
+      <c r="W14" s="109"/>
+      <c r="X14" s="109"/>
+      <c r="Y14" s="109"/>
+      <c r="Z14" s="109"/>
+      <c r="AA14" s="109"/>
+      <c r="AB14" s="109"/>
+      <c r="AC14" s="109"/>
+      <c r="AD14" s="109"/>
+      <c r="AE14" s="109"/>
+      <c r="AF14" s="109"/>
+      <c r="AG14" s="109"/>
+      <c r="AH14" s="109"/>
+      <c r="AI14" s="109"/>
+      <c r="AJ14" s="109"/>
+      <c r="AK14" s="109"/>
+      <c r="AL14" s="109"/>
+      <c r="AM14" s="109"/>
+      <c r="AN14" s="109"/>
+      <c r="AO14" s="109"/>
+      <c r="AP14" s="109"/>
+      <c r="AQ14" s="109"/>
+      <c r="AR14" s="110"/>
       <c r="AS14" s="25"/>
       <c r="AT14" s="25"/>
       <c r="AU14" s="25" t="s">
@@ -4086,85 +4090,85 @@
       </c>
     </row>
     <row r="15" spans="1:47" s="1" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="104"/>
+      <c r="A15" s="117"/>
       <c r="B15" s="115"/>
       <c r="C15" s="116"/>
-      <c r="D15" s="104"/>
-      <c r="E15" s="65" t="s">
+      <c r="D15" s="117"/>
+      <c r="E15" s="114" t="s">
         <v>88</v>
       </c>
-      <c r="F15" s="65"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="65"/>
-      <c r="I15" s="65" t="s">
+      <c r="F15" s="114"/>
+      <c r="G15" s="114"/>
+      <c r="H15" s="114"/>
+      <c r="I15" s="114" t="s">
         <v>89</v>
       </c>
-      <c r="J15" s="65"/>
-      <c r="K15" s="65"/>
-      <c r="L15" s="65"/>
-      <c r="M15" s="97" t="s">
+      <c r="J15" s="114"/>
+      <c r="K15" s="114"/>
+      <c r="L15" s="114"/>
+      <c r="M15" s="68" t="s">
         <v>90</v>
       </c>
-      <c r="N15" s="97"/>
-      <c r="O15" s="97"/>
-      <c r="P15" s="97"/>
-      <c r="Q15" s="65" t="s">
+      <c r="N15" s="68"/>
+      <c r="O15" s="68"/>
+      <c r="P15" s="68"/>
+      <c r="Q15" s="114" t="s">
         <v>91</v>
       </c>
-      <c r="R15" s="65"/>
-      <c r="S15" s="65"/>
-      <c r="T15" s="65"/>
-      <c r="U15" s="65" t="s">
+      <c r="R15" s="114"/>
+      <c r="S15" s="114"/>
+      <c r="T15" s="114"/>
+      <c r="U15" s="114" t="s">
         <v>92</v>
       </c>
-      <c r="V15" s="65"/>
-      <c r="W15" s="65"/>
-      <c r="X15" s="65"/>
-      <c r="Y15" s="65" t="s">
+      <c r="V15" s="114"/>
+      <c r="W15" s="114"/>
+      <c r="X15" s="114"/>
+      <c r="Y15" s="114" t="s">
         <v>93</v>
       </c>
-      <c r="Z15" s="65"/>
-      <c r="AA15" s="65"/>
-      <c r="AB15" s="65"/>
-      <c r="AC15" s="65" t="s">
+      <c r="Z15" s="114"/>
+      <c r="AA15" s="114"/>
+      <c r="AB15" s="114"/>
+      <c r="AC15" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="AD15" s="65"/>
-      <c r="AE15" s="65"/>
-      <c r="AF15" s="65"/>
-      <c r="AG15" s="65" t="s">
+      <c r="AD15" s="114"/>
+      <c r="AE15" s="114"/>
+      <c r="AF15" s="114"/>
+      <c r="AG15" s="114" t="s">
         <v>95</v>
       </c>
-      <c r="AH15" s="65"/>
-      <c r="AI15" s="65"/>
-      <c r="AJ15" s="65"/>
-      <c r="AK15" s="65" t="s">
+      <c r="AH15" s="114"/>
+      <c r="AI15" s="114"/>
+      <c r="AJ15" s="114"/>
+      <c r="AK15" s="114" t="s">
         <v>96</v>
       </c>
-      <c r="AL15" s="65"/>
-      <c r="AM15" s="65"/>
-      <c r="AN15" s="65"/>
-      <c r="AO15" s="65" t="s">
+      <c r="AL15" s="114"/>
+      <c r="AM15" s="114"/>
+      <c r="AN15" s="114"/>
+      <c r="AO15" s="114" t="s">
         <v>97</v>
       </c>
-      <c r="AP15" s="65"/>
-      <c r="AQ15" s="65"/>
-      <c r="AR15" s="65"/>
-      <c r="AS15" s="106" t="s">
+      <c r="AP15" s="114"/>
+      <c r="AQ15" s="114"/>
+      <c r="AR15" s="114"/>
+      <c r="AS15" s="104" t="s">
         <v>10</v>
       </c>
-      <c r="AT15" s="106" t="s">
+      <c r="AT15" s="104" t="s">
         <v>11</v>
       </c>
-      <c r="AU15" s="106" t="s">
+      <c r="AU15" s="104" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:47" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="104"/>
+      <c r="A16" s="117"/>
       <c r="B16" s="115"/>
       <c r="C16" s="116"/>
-      <c r="D16" s="104"/>
+      <c r="D16" s="117"/>
       <c r="E16" s="29" t="s">
         <v>98</v>
       </c>
@@ -4285,9 +4289,9 @@
       <c r="AR16" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="AS16" s="108"/>
-      <c r="AT16" s="108"/>
-      <c r="AU16" s="107"/>
+      <c r="AS16" s="106"/>
+      <c r="AT16" s="106"/>
+      <c r="AU16" s="105"/>
     </row>
     <row r="17" spans="1:47" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
@@ -4300,28 +4304,30 @@
         <v>131</v>
       </c>
       <c r="D17" s="17"/>
-      <c r="E17" s="20">
+      <c r="I17" s="20">
         <v>25</v>
       </c>
-      <c r="F17" s="17">
-        <v>0</v>
-      </c>
-      <c r="G17" s="20">
+      <c r="J17" s="17">
+        <v>0</v>
+      </c>
+      <c r="K17" s="20">
         <v>5</v>
       </c>
-      <c r="H17" s="17">
-        <v>0</v>
-      </c>
-      <c r="I17" s="20"/>
-      <c r="J17" s="17">
+      <c r="L17" s="17">
+        <v>0</v>
+      </c>
+      <c r="M17" s="20">
+        <v>20</v>
+      </c>
+      <c r="N17" s="17">
         <v>1</v>
       </c>
-      <c r="K17" s="20"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="20"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="20"/>
-      <c r="P17" s="17"/>
+      <c r="O17" s="20">
+        <v>5</v>
+      </c>
+      <c r="P17" s="17">
+        <v>0</v>
+      </c>
       <c r="Q17" s="20"/>
       <c r="R17" s="17"/>
       <c r="S17" s="20"/>
@@ -4367,26 +4373,30 @@
         <v>132</v>
       </c>
       <c r="D18" s="17"/>
-      <c r="E18" s="20">
+      <c r="I18" s="20">
         <v>25</v>
       </c>
-      <c r="F18" s="17">
-        <v>0</v>
-      </c>
-      <c r="G18" s="20">
+      <c r="J18" s="17">
+        <v>0</v>
+      </c>
+      <c r="K18" s="20">
         <v>5</v>
       </c>
-      <c r="H18" s="17">
-        <v>0</v>
-      </c>
-      <c r="I18" s="20"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="20"/>
-      <c r="P18" s="17"/>
+      <c r="L18" s="17">
+        <v>0</v>
+      </c>
+      <c r="M18" s="20">
+        <v>20</v>
+      </c>
+      <c r="N18" s="17">
+        <v>0</v>
+      </c>
+      <c r="O18" s="20">
+        <v>5</v>
+      </c>
+      <c r="P18" s="17">
+        <v>0</v>
+      </c>
       <c r="Q18" s="20"/>
       <c r="R18" s="17"/>
       <c r="S18" s="20"/>
@@ -6883,7 +6893,7 @@
       </c>
       <c r="E69" s="34">
         <f>SUM(E17:E68)</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F69" s="34">
         <f>SUM(F17:F68)</f>
@@ -6891,39 +6901,39 @@
       </c>
       <c r="G69" s="34">
         <f t="shared" ref="G69:AR69" si="0">SUM(G17:G68)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H69" s="34">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I69" s="34">
+        <f>SUM(I17:I68)</f>
+        <v>50</v>
+      </c>
+      <c r="J69" s="34">
+        <f>SUM(J17:J68)</f>
+        <v>0</v>
+      </c>
+      <c r="K69" s="34">
+        <f>SUM(K17:K68)</f>
+        <v>10</v>
+      </c>
+      <c r="L69" s="34">
+        <f>SUM(L17:L68)</f>
+        <v>0</v>
+      </c>
+      <c r="M69" s="34">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J69" s="34">
+        <v>40</v>
+      </c>
+      <c r="N69" s="34">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K69" s="34">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L69" s="34">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M69" s="34">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="N69" s="34">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="O69" s="34">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P69" s="34">
         <f t="shared" si="0"/>
@@ -7047,6 +7057,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AK15:AN15"/>
+    <mergeCell ref="AO15:AR15"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="U15:X15"/>
+    <mergeCell ref="Y15:AB15"/>
+    <mergeCell ref="AC15:AF15"/>
+    <mergeCell ref="AG15:AJ15"/>
+    <mergeCell ref="E15:H15"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="AU15:AU16"/>
     <mergeCell ref="AS15:AS16"/>
     <mergeCell ref="AT15:AT16"/>
@@ -7063,20 +7087,6 @@
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="I15:L15"/>
     <mergeCell ref="M15:P15"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="AK15:AN15"/>
-    <mergeCell ref="AO15:AR15"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="U15:X15"/>
-    <mergeCell ref="Y15:AB15"/>
-    <mergeCell ref="AC15:AF15"/>
-    <mergeCell ref="AG15:AJ15"/>
-    <mergeCell ref="E15:H15"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="A13">
@@ -7122,7 +7132,7 @@
       <c r="M1" s="3"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="102" t="s">
         <v>26</v>
       </c>
       <c r="B2" s="47"/>
@@ -7139,7 +7149,7 @@
       <c r="M2" s="47"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="67"/>
+      <c r="A3" s="99"/>
       <c r="B3" s="47"/>
       <c r="C3" s="47"/>
       <c r="D3" s="47"/>
@@ -7154,7 +7164,7 @@
       <c r="M3" s="47"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="67"/>
+      <c r="A4" s="99"/>
       <c r="B4" s="7"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -7167,18 +7177,18 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="48"/>
-      <c r="B7" s="65" t="s">
+      <c r="B7" s="114" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="65"/>
-      <c r="I7" s="65"/>
-      <c r="J7" s="65"/>
-      <c r="K7" s="65"/>
+      <c r="C7" s="114"/>
+      <c r="D7" s="114"/>
+      <c r="E7" s="114"/>
+      <c r="F7" s="114"/>
+      <c r="G7" s="114"/>
+      <c r="H7" s="114"/>
+      <c r="I7" s="114"/>
+      <c r="J7" s="114"/>
+      <c r="K7" s="114"/>
       <c r="L7" s="17"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -7254,7 +7264,9 @@
       <c r="C10" s="20">
         <v>3.5</v>
       </c>
-      <c r="D10" s="17"/>
+      <c r="D10" s="17">
+        <v>4</v>
+      </c>
       <c r="E10" s="20"/>
       <c r="F10" s="17"/>
       <c r="G10" s="20"/>
@@ -7264,7 +7276,7 @@
       <c r="K10" s="20"/>
       <c r="L10" s="34">
         <f t="shared" ref="L10:L15" si="0">SUM(B10:K10)</f>
-        <v>5.25</v>
+        <v>9.25</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -7277,7 +7289,7 @@
       <c r="C11" s="20">
         <v>3.75</v>
       </c>
-      <c r="D11" s="117">
+      <c r="D11" s="65">
         <v>6.75</v>
       </c>
       <c r="E11" s="20"/>
@@ -7497,7 +7509,7 @@
       </c>
       <c r="B3">
         <f>SUM('General Tasks'!E30,'General Tasks'!G30,'General Tasks'!I30,'General Tasks'!K30,'General Tasks'!M30,'General Tasks'!O30,'General Tasks'!Q30,'General Tasks'!S30,'General Tasks'!U30,'General Tasks'!W30,Requirements!F69,Requirements!H69,Requirements!J69,Requirements!L69,Requirements!N69,Requirements!P69,Requirements!R69,Requirements!T69,Requirements!V69,Requirements!X69,Requirements!Z69,Requirements!AB69,Requirements!AD69,Requirements!AF69,Requirements!AH69,Requirements!AJ69,Requirements!AL69,Requirements!AN69,Requirements!AP69,Requirements!AR69)</f>
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D3" s="40"/>
       <c r="P3">
@@ -7515,7 +7527,7 @@
       </c>
       <c r="B4">
         <f>B2-B3</f>
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C4" t="str">
         <f>IF(B4&gt;=0,"within budget","over budget")</f>
@@ -7537,7 +7549,7 @@
       </c>
       <c r="B5">
         <f>(('General Tasks'!C9)-B3)</f>
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C5" t="str">
         <f>IF(B5&gt;=0,"within budget","over budget")</f>
@@ -7551,7 +7563,7 @@
       </c>
       <c r="B6">
         <f>(SUM('General Tasks'!H30,Requirements!M69,Requirements!O69) - (B3))</f>
-        <v>155</v>
+        <v>202</v>
       </c>
       <c r="C6" t="str">
         <f>IF(B6&gt;=0,"within estimate","over estimate")</f>
@@ -7575,7 +7587,7 @@
       </c>
       <c r="B7" s="43">
         <f>(SUM('General Tasks'!P30,Requirements!AC69,Requirements!AE69) - (B4))</f>
-        <v>-285</v>
+        <v>-282</v>
       </c>
       <c r="C7" s="43" t="str">
         <f>IF(B7&gt;=0,"within estimate","over estimate")</f>

</xml_diff>